<commit_message>
feat: add Excel parser with tests
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample_data.xlsx
+++ b/tests/fixtures/sample_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>总工时</t>
+          <t>总耗时</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -434,7 +434,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>工时</t>
+          <t>耗时</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -444,7 +444,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>明细工时</t>
+          <t>耗时.1</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -454,7 +454,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>每日工时</t>
+          <t>耗时.2</t>
         </is>
       </c>
     </row>
@@ -465,53 +465,63 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>项目A</t>
+          <t>泰擎II期</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>需求分析</t>
+          <t>完成学生画像8维度设计</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-03-01:完成需求文档</t>
+          <t>2026-03-23:完成学生画像8维度设计</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>张三</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>泰擎II期</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>开发工作</t>
+          <t>OCR识别功能开发</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-03-02:完成API开发</t>
+          <t>2026-03-24:OCR识别功能开发</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -521,59 +531,31 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>项目B</t>
+          <t>泰擎II期</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>测试工作</t>
+          <t>形成性评价系统优化</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-03-01:编写测试用例</t>
+          <t>2026-03-23:形成性评价系统优化</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>项目C</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>20</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>前端开发</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>20</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-03-03:完成页面开发</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>